<commit_message>
support only key_output weights
</commit_message>
<xml_diff>
--- a/src/vlinder/data/DSM/xlsx/DSM.xlsx
+++ b/src/vlinder/data/DSM/xlsx/DSM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10211"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lheringa001\Desktop\RBS_opensource\trbs_dsm\model\data\DSM\xlsx\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tdijk004/Documents/Tooling/tRBS/open source/trbs/src/vlinder/data/DSM/xlsx/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47E91D93-C97C-46C5-A426-D7D1DDD1917D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A6E7839-DA64-9848-80BC-1D1340E173C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="configurations" sheetId="1" r:id="rId1"/>
@@ -416,8 +416,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="164" formatCode="0.0000"/>
+    <numFmt numFmtId="164" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
   </numFmts>
   <fonts count="10" x14ac:knownFonts="1">
     <font>
@@ -431,6 +431,7 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -443,6 +444,7 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -460,17 +462,20 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -545,9 +550,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -581,8 +586,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -595,17 +599,13 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Komma" xfId="1" builtinId="3"/>
+    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -906,12 +906,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -919,12 +919,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -935,20 +935,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:I10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="37.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="37.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.83203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -977,248 +977,239 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
         <v>31</v>
       </c>
       <c r="B2" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="13">
+      <c r="C2">
         <v>0</v>
       </c>
       <c r="D2" s="3">
         <v>1</v>
       </c>
-      <c r="E2" s="13">
-        <v>0</v>
-      </c>
-      <c r="F2" s="13">
-        <v>1</v>
-      </c>
-      <c r="G2" s="14">
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2" s="13">
         <v>-41400000</v>
       </c>
-      <c r="H2" s="14">
+      <c r="H2" s="13">
         <v>30000000</v>
       </c>
-      <c r="I2" s="13"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="12" t="s">
         <v>32</v>
       </c>
       <c r="B3" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="13">
+      <c r="C3">
         <v>0</v>
       </c>
       <c r="D3" s="3">
         <v>1</v>
       </c>
-      <c r="E3" s="13">
-        <v>1</v>
-      </c>
-      <c r="F3" s="13">
-        <v>1</v>
-      </c>
-      <c r="G3" s="14">
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3" s="13">
         <v>5734800</v>
       </c>
-      <c r="H3" s="14">
+      <c r="H3" s="13">
         <v>8389800</v>
       </c>
-      <c r="I3" s="13"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="12" t="s">
         <v>33</v>
       </c>
       <c r="B4" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="13">
+      <c r="C4">
         <v>0</v>
       </c>
       <c r="D4" s="3">
         <v>0</v>
       </c>
-      <c r="E4" s="13">
-        <v>0</v>
-      </c>
-      <c r="F4" s="13">
-        <v>1</v>
-      </c>
-      <c r="G4" s="14">
-        <v>0</v>
-      </c>
-      <c r="H4" s="14">
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4" s="13">
+        <v>0</v>
+      </c>
+      <c r="H4" s="13">
         <v>0.1</v>
       </c>
-      <c r="I4" s="13"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="12" t="s">
         <v>34</v>
       </c>
       <c r="B5" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="13">
+      <c r="C5">
         <v>0</v>
       </c>
       <c r="D5" s="3">
         <v>0</v>
       </c>
-      <c r="E5" s="13">
-        <v>0</v>
-      </c>
-      <c r="F5" s="13">
-        <v>1</v>
-      </c>
-      <c r="G5" s="14">
-        <v>0</v>
-      </c>
-      <c r="H5" s="14">
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5" s="13">
+        <v>0</v>
+      </c>
+      <c r="H5" s="13">
         <v>3988.3999999999942</v>
       </c>
-      <c r="I5" s="13"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" s="12" t="s">
         <v>35</v>
       </c>
       <c r="B6" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="13">
+      <c r="C6">
         <v>0</v>
       </c>
       <c r="D6" s="3">
         <v>1</v>
       </c>
-      <c r="E6" s="13">
-        <v>0</v>
-      </c>
-      <c r="F6" s="13">
-        <v>1</v>
-      </c>
-      <c r="G6" s="14">
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6" s="13">
         <v>39884</v>
       </c>
-      <c r="H6" s="14">
+      <c r="H6" s="13">
         <v>39884</v>
       </c>
-      <c r="I6" s="13"/>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" s="12" t="s">
         <v>36</v>
       </c>
       <c r="B7" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="13">
+      <c r="C7">
         <v>0</v>
       </c>
       <c r="D7" s="3">
         <v>0</v>
       </c>
-      <c r="E7" s="13">
-        <v>0</v>
-      </c>
-      <c r="F7" s="13">
-        <v>1</v>
-      </c>
-      <c r="G7" s="14">
-        <v>0</v>
-      </c>
-      <c r="H7" s="14">
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7" s="13">
+        <v>0</v>
+      </c>
+      <c r="H7" s="13">
         <v>1.73</v>
       </c>
-      <c r="I7" s="13"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" s="12" t="s">
         <v>37</v>
       </c>
       <c r="B8" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="13">
+      <c r="C8">
         <v>0</v>
       </c>
       <c r="D8" s="3">
         <v>0</v>
       </c>
-      <c r="E8" s="13">
-        <v>0</v>
-      </c>
-      <c r="F8" s="13">
-        <v>1</v>
-      </c>
-      <c r="G8" s="14">
-        <v>0</v>
-      </c>
-      <c r="H8" s="14">
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="G8" s="13">
+        <v>0</v>
+      </c>
+      <c r="H8" s="13">
         <v>1.1244999999999998</v>
       </c>
-      <c r="I8" s="13"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" s="12" t="s">
         <v>38</v>
       </c>
       <c r="B9" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="13">
+      <c r="C9">
         <v>0</v>
       </c>
       <c r="D9" s="3">
         <v>0</v>
       </c>
-      <c r="E9" s="13">
-        <v>0</v>
-      </c>
-      <c r="F9" s="13">
-        <v>1</v>
-      </c>
-      <c r="G9" s="14">
-        <v>0</v>
-      </c>
-      <c r="H9" s="14">
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9" s="13">
+        <v>0</v>
+      </c>
+      <c r="H9" s="13">
         <v>0.17300000000000001</v>
       </c>
-      <c r="I9" s="13"/>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" s="12" t="s">
         <v>39</v>
       </c>
       <c r="B10" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="13">
+      <c r="C10">
         <v>0</v>
       </c>
       <c r="D10" s="3">
         <v>0</v>
       </c>
-      <c r="E10" s="13">
-        <v>0</v>
-      </c>
-      <c r="F10" s="13">
-        <v>1</v>
-      </c>
-      <c r="G10" s="14">
-        <v>0</v>
-      </c>
-      <c r="H10" s="14">
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>1</v>
+      </c>
+      <c r="G10" s="13">
+        <v>0</v>
+      </c>
+      <c r="H10" s="13">
         <v>845540.79999999877</v>
       </c>
-      <c r="I10" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1229,13 +1220,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F43"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>15</v>
       </c>
@@ -1246,7 +1237,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>40</v>
       </c>
@@ -1257,7 +1248,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>43</v>
       </c>
@@ -1268,7 +1259,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>41</v>
       </c>
@@ -1279,7 +1270,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>42</v>
       </c>
@@ -1290,7 +1281,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>111</v>
       </c>
@@ -1301,7 +1292,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>110</v>
       </c>
@@ -1312,7 +1303,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>112</v>
       </c>
@@ -1323,7 +1314,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>40</v>
       </c>
@@ -1334,7 +1325,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>43</v>
       </c>
@@ -1345,7 +1336,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>41</v>
       </c>
@@ -1356,7 +1347,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>42</v>
       </c>
@@ -1367,7 +1358,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>111</v>
       </c>
@@ -1378,7 +1369,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>110</v>
       </c>
@@ -1389,7 +1380,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>112</v>
       </c>
@@ -1400,7 +1391,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>40</v>
       </c>
@@ -1411,7 +1402,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>43</v>
       </c>
@@ -1422,7 +1413,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>41</v>
       </c>
@@ -1433,7 +1424,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>42</v>
       </c>
@@ -1444,7 +1435,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>111</v>
       </c>
@@ -1455,7 +1446,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>110</v>
       </c>
@@ -1466,7 +1457,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>112</v>
       </c>
@@ -1477,7 +1468,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>40</v>
       </c>
@@ -1488,7 +1479,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>43</v>
       </c>
@@ -1499,7 +1490,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>41</v>
       </c>
@@ -1510,7 +1501,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
         <v>42</v>
       </c>
@@ -1521,7 +1512,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
         <v>111</v>
       </c>
@@ -1532,7 +1523,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>110</v>
       </c>
@@ -1543,7 +1534,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
         <v>112</v>
       </c>
@@ -1554,7 +1545,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
         <v>40</v>
       </c>
@@ -1565,7 +1556,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
         <v>43</v>
       </c>
@@ -1576,7 +1567,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
         <v>41</v>
       </c>
@@ -1587,7 +1578,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
         <v>42</v>
       </c>
@@ -1598,7 +1589,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
         <v>111</v>
       </c>
@@ -1609,7 +1600,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
         <v>110</v>
       </c>
@@ -1620,7 +1611,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
         <v>112</v>
       </c>
@@ -1631,7 +1622,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
         <v>40</v>
       </c>
@@ -1643,7 +1634,7 @@
       </c>
       <c r="F37" s="10"/>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
         <v>43</v>
       </c>
@@ -1655,7 +1646,7 @@
       </c>
       <c r="F38" s="10"/>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
         <v>41</v>
       </c>
@@ -1667,7 +1658,7 @@
       </c>
       <c r="F39" s="10"/>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
         <v>42</v>
       </c>
@@ -1679,7 +1670,7 @@
       </c>
       <c r="F40" s="10"/>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
         <v>111</v>
       </c>
@@ -1691,7 +1682,7 @@
       </c>
       <c r="F41" s="10"/>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
         <v>110</v>
       </c>
@@ -1703,7 +1694,7 @@
       </c>
       <c r="F42" s="10"/>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
         <v>112</v>
       </c>
@@ -1726,14 +1717,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:C22"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="25.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>17</v>
       </c>
@@ -1744,7 +1735,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
         <v>48</v>
       </c>
@@ -1755,7 +1746,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>49</v>
       </c>
@@ -1766,7 +1757,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
         <v>50</v>
       </c>
@@ -1777,7 +1768,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
         <v>51</v>
       </c>
@@ -1788,7 +1779,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
         <v>52</v>
       </c>
@@ -1799,7 +1790,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
         <v>53</v>
       </c>
@@ -1810,7 +1801,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
         <v>54</v>
       </c>
@@ -1821,7 +1812,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
         <v>48</v>
       </c>
@@ -1832,7 +1823,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
         <v>49</v>
       </c>
@@ -1843,7 +1834,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
         <v>50</v>
       </c>
@@ -1854,7 +1845,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
         <v>51</v>
       </c>
@@ -1865,7 +1856,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" s="6" t="s">
         <v>52</v>
       </c>
@@ -1876,7 +1867,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="6" t="s">
         <v>53</v>
       </c>
@@ -1887,7 +1878,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="6" t="s">
         <v>54</v>
       </c>
@@ -1898,7 +1889,7 @@
         <v>0.35</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="6" t="s">
         <v>48</v>
       </c>
@@ -1909,7 +1900,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="6" t="s">
         <v>49</v>
       </c>
@@ -1920,7 +1911,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="6" t="s">
         <v>50</v>
       </c>
@@ -1931,7 +1922,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="6" t="s">
         <v>51</v>
       </c>
@@ -1942,7 +1933,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="6" t="s">
         <v>52</v>
       </c>
@@ -1953,7 +1944,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="6" t="s">
         <v>53</v>
       </c>
@@ -1964,7 +1955,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="6" t="s">
         <v>54</v>
       </c>
@@ -1983,12 +1974,12 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:B71"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="61.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="61.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>19</v>
       </c>
@@ -1996,7 +1987,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>57</v>
       </c>
@@ -2004,7 +1995,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>58</v>
       </c>
@@ -2012,7 +2003,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>59</v>
       </c>
@@ -2020,7 +2011,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>60</v>
       </c>
@@ -2028,7 +2019,7 @@
         <v>0.67600000000000005</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>61</v>
       </c>
@@ -2036,7 +2027,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>62</v>
       </c>
@@ -2044,7 +2035,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>63</v>
       </c>
@@ -2052,7 +2043,7 @@
         <v>0.13</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>64</v>
       </c>
@@ -2060,7 +2051,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>65</v>
       </c>
@@ -2068,7 +2059,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>66</v>
       </c>
@@ -2076,7 +2067,7 @@
         <v>1.7299999999999999E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>67</v>
       </c>
@@ -2084,7 +2075,7 @@
         <v>1.7299999999999999E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>68</v>
       </c>
@@ -2092,7 +2083,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>69</v>
       </c>
@@ -2100,7 +2091,7 @@
         <v>0.78</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>70</v>
       </c>
@@ -2108,172 +2099,172 @@
         <v>40000000</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" s="7"/>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A17" s="7"/>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A18" s="7"/>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" s="7"/>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A20" s="7"/>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A21" s="7"/>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A22" s="7"/>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A23" s="7"/>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A24" s="7"/>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A25" s="7"/>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A26" s="7"/>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A27" s="7"/>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A28" s="7"/>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A29" s="7"/>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A30" s="7"/>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A31" s="7"/>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A32" s="7"/>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A33" s="7"/>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A34" s="7"/>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A35" s="7"/>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A36" s="7"/>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A37" s="7"/>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A38" s="7"/>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A39" s="7"/>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A40" s="7"/>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A41" s="7"/>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A42" s="7"/>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A43" s="7"/>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A44" s="7"/>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A45" s="7"/>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A46" s="7"/>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A47" s="7"/>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A48" s="7"/>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A49" s="7"/>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A50" s="7"/>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A51" s="7"/>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A52" s="7"/>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A53" s="7"/>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A54" s="7"/>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A55" s="7"/>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A56" s="7"/>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A57" s="7"/>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A58" s="7"/>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A59" s="7"/>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A60" s="7"/>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A61" s="7"/>
     </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A62" s="7"/>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A63" s="7"/>
     </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A64" s="7"/>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A65" s="7"/>
     </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A66" s="7"/>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A67" s="7"/>
     </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A68" s="7"/>
     </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A69" s="7"/>
     </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A70" s="7"/>
     </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A71" s="7"/>
     </row>
   </sheetData>
@@ -2284,19 +2275,19 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:H72"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="40.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="37.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="67.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="40.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="37.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="67.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>20</v>
       </c>
@@ -2322,7 +2313,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="11" t="s">
         <v>71</v>
       </c>
@@ -2336,7 +2327,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="11" t="s">
         <v>71</v>
       </c>
@@ -2350,7 +2341,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="11" t="s">
         <v>72</v>
       </c>
@@ -2364,7 +2355,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="11" t="s">
         <v>73</v>
       </c>
@@ -2378,49 +2369,49 @@
         <v>118</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="B6" s="21" t="s">
+      <c r="B6" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="C6" s="21" t="s">
+      <c r="C6" s="11" t="s">
         <v>73</v>
       </c>
       <c r="D6" s="11" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="11" t="s">
         <v>124</v>
       </c>
       <c r="B7" s="11">
         <v>1</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" t="s">
         <v>54</v>
       </c>
       <c r="D7" s="11" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="11" t="s">
         <v>124</v>
       </c>
       <c r="B8" s="11">
         <v>0</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C8" t="s">
         <v>53</v>
       </c>
-      <c r="D8" s="18" t="s">
+      <c r="D8" s="17" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="11" t="s">
         <v>74</v>
       </c>
@@ -2434,7 +2425,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="11" t="s">
         <v>103</v>
       </c>
@@ -2448,21 +2439,21 @@
         <v>28</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B11" s="11" t="s">
         <v>103</v>
       </c>
-      <c r="C11" s="18" t="s">
+      <c r="C11" s="17" t="s">
         <v>124</v>
       </c>
       <c r="D11" s="11" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="11" t="s">
         <v>75</v>
       </c>
@@ -2476,7 +2467,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="11" t="s">
         <v>76</v>
       </c>
@@ -2490,7 +2481,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="11" t="s">
         <v>77</v>
       </c>
@@ -2504,7 +2495,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" s="11" t="s">
         <v>78</v>
       </c>
@@ -2518,7 +2509,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" s="11" t="s">
         <v>79</v>
       </c>
@@ -2532,7 +2523,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="11" t="s">
         <v>80</v>
       </c>
@@ -2546,7 +2537,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" s="11" t="s">
         <v>81</v>
       </c>
@@ -2560,7 +2551,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="11" t="s">
         <v>82</v>
       </c>
@@ -2574,7 +2565,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" s="11" t="s">
         <v>83</v>
       </c>
@@ -2588,7 +2579,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A21" s="11" t="s">
         <v>84</v>
       </c>
@@ -2602,7 +2593,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A22" s="11" t="s">
         <v>85</v>
       </c>
@@ -2616,7 +2607,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" s="11" t="s">
         <v>86</v>
       </c>
@@ -2630,7 +2621,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" s="11" t="s">
         <v>87</v>
       </c>
@@ -2644,7 +2635,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A25" s="11" t="s">
         <v>88</v>
       </c>
@@ -2658,7 +2649,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A26" s="11" t="s">
         <v>88</v>
       </c>
@@ -2672,7 +2663,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" s="11" t="s">
         <v>89</v>
       </c>
@@ -2686,7 +2677,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A28" s="11" t="s">
         <v>90</v>
       </c>
@@ -2700,7 +2691,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A29" s="11" t="s">
         <v>91</v>
       </c>
@@ -2714,7 +2705,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A30" s="11" t="s">
         <v>91</v>
       </c>
@@ -2728,7 +2719,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A31" s="11" t="s">
         <v>125</v>
       </c>
@@ -2742,7 +2733,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A32" s="11" t="s">
         <v>125</v>
       </c>
@@ -2756,7 +2747,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A33" s="11" t="s">
         <v>125</v>
       </c>
@@ -2770,21 +2761,21 @@
         <v>121</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A34" s="11" t="s">
         <v>93</v>
       </c>
       <c r="B34" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="C34" s="20" t="s">
+      <c r="C34" s="18" t="s">
         <v>125</v>
       </c>
       <c r="D34" s="11" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A35" s="11" t="s">
         <v>94</v>
       </c>
@@ -2798,7 +2789,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A36" s="11" t="s">
         <v>104</v>
       </c>
@@ -2812,7 +2803,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A37" s="11" t="s">
         <v>104</v>
       </c>
@@ -2826,7 +2817,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A38" s="11" t="s">
         <v>105</v>
       </c>
@@ -2840,7 +2831,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A39" s="11" t="s">
         <v>106</v>
       </c>
@@ -2854,7 +2845,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A40" s="11" t="s">
         <v>106</v>
       </c>
@@ -2868,7 +2859,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A41" s="11" t="s">
         <v>107</v>
       </c>
@@ -2882,7 +2873,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A42" s="11" t="s">
         <v>95</v>
       </c>
@@ -2896,7 +2887,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A43" s="11" t="s">
         <v>95</v>
       </c>
@@ -2910,7 +2901,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A44" s="11" t="s">
         <v>96</v>
       </c>
@@ -2924,7 +2915,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A45" s="11" t="s">
         <v>35</v>
       </c>
@@ -2938,7 +2929,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A46" s="11" t="s">
         <v>97</v>
       </c>
@@ -2952,7 +2943,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A47" s="11" t="s">
         <v>32</v>
       </c>
@@ -2966,7 +2957,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A48" s="11" t="s">
         <v>32</v>
       </c>
@@ -2980,7 +2971,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A49" s="11" t="s">
         <v>32</v>
       </c>
@@ -2994,7 +2985,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A50" s="11" t="s">
         <v>33</v>
       </c>
@@ -3008,7 +2999,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A51" s="11" t="s">
         <v>33</v>
       </c>
@@ -3022,7 +3013,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A52" s="11" t="s">
         <v>98</v>
       </c>
@@ -3036,7 +3027,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A53" s="11" t="s">
         <v>34</v>
       </c>
@@ -3050,7 +3041,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A54" s="11" t="s">
         <v>34</v>
       </c>
@@ -3064,21 +3055,21 @@
         <v>120</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A55" s="16" t="s">
+    <row r="55" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A55" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="B55" s="16" t="s">
+      <c r="B55" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="C55" s="16" t="s">
+      <c r="C55" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="D55" s="16" t="s">
+      <c r="D55" s="15" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A56" s="11" t="s">
         <v>100</v>
       </c>
@@ -3092,149 +3083,149 @@
         <v>115</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A57" s="16" t="s">
+    <row r="57" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A57" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="B57" s="16" t="s">
+      <c r="B57" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="C57" s="16" t="s">
+      <c r="C57" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="D57" s="16" t="s">
+      <c r="D57" s="15" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A58" s="16" t="s">
+    <row r="58" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A58" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="B58" s="16" t="s">
+      <c r="B58" s="15" t="s">
         <v>61</v>
       </c>
-      <c r="C58" s="16" t="s">
+      <c r="C58" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="D58" s="16" t="s">
+      <c r="D58" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="E58" s="17"/>
-      <c r="F58" s="17"/>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A59" s="16" t="s">
+      <c r="E58" s="16"/>
+      <c r="F58" s="16"/>
+    </row>
+    <row r="59" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A59" s="15" t="s">
         <v>122</v>
       </c>
-      <c r="B59" s="16">
-        <v>1</v>
-      </c>
-      <c r="C59" s="16" t="s">
+      <c r="B59" s="15">
+        <v>1</v>
+      </c>
+      <c r="C59" s="15" t="s">
         <v>61</v>
       </c>
-      <c r="D59" s="16" t="s">
+      <c r="D59" s="15" t="s">
         <v>120</v>
       </c>
-      <c r="E59" s="17"/>
-      <c r="F59" s="17"/>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A60" s="16" t="s">
+      <c r="E59" s="16"/>
+      <c r="F59" s="16"/>
+    </row>
+    <row r="60" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A60" s="15" t="s">
         <v>123</v>
       </c>
-      <c r="B60" s="16">
-        <v>1</v>
-      </c>
-      <c r="C60" s="16" t="s">
+      <c r="B60" s="15">
+        <v>1</v>
+      </c>
+      <c r="C60" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="D60" s="16" t="s">
+      <c r="D60" s="15" t="s">
         <v>120</v>
       </c>
-      <c r="E60" s="17"/>
-      <c r="F60" s="17"/>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A61" s="16" t="s">
+      <c r="E60" s="16"/>
+      <c r="F60" s="16"/>
+    </row>
+    <row r="61" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A61" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="B61" s="16" t="s">
+      <c r="B61" s="15" t="s">
         <v>61</v>
       </c>
-      <c r="C61" s="16" t="s">
+      <c r="C61" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="D61" s="16" t="s">
+      <c r="D61" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="E61" s="17"/>
-      <c r="F61" s="17"/>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A62" s="16" t="s">
+      <c r="E61" s="16"/>
+      <c r="F61" s="16"/>
+    </row>
+    <row r="62" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A62" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="B62" s="16" t="s">
+      <c r="B62" s="15" t="s">
         <v>122</v>
       </c>
-      <c r="C62" s="16" t="s">
+      <c r="C62" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="D62" s="16" t="s">
+      <c r="D62" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="E62" s="17"/>
-      <c r="F62" s="17"/>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A63" s="16" t="s">
+      <c r="E62" s="16"/>
+      <c r="F62" s="16"/>
+    </row>
+    <row r="63" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A63" s="15" t="s">
         <v>109</v>
       </c>
-      <c r="B63" s="16" t="s">
+      <c r="B63" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="C63" s="16" t="s">
+      <c r="C63" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="D63" s="16" t="s">
+      <c r="D63" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="E63" s="17"/>
-      <c r="F63" s="17"/>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A64" s="16" t="s">
+      <c r="E63" s="16"/>
+      <c r="F63" s="16"/>
+    </row>
+    <row r="64" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A64" s="15" t="s">
         <v>109</v>
       </c>
-      <c r="B64" s="16" t="s">
+      <c r="B64" s="15" t="s">
         <v>123</v>
       </c>
-      <c r="C64" s="16" t="s">
+      <c r="C64" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="D64" s="16" t="s">
+      <c r="D64" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="E64" s="17"/>
-      <c r="F64" s="17"/>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A65" s="16" t="s">
+      <c r="E64" s="16"/>
+      <c r="F64" s="16"/>
+    </row>
+    <row r="65" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A65" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="B65" s="16" t="s">
+      <c r="B65" s="15" t="s">
         <v>109</v>
       </c>
-      <c r="C65" s="16" t="s">
+      <c r="C65" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="D65" s="16" t="s">
+      <c r="D65" s="15" t="s">
         <v>120</v>
       </c>
-      <c r="E65" s="17"/>
-      <c r="F65" s="17"/>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E65" s="16"/>
+      <c r="F65" s="16"/>
+    </row>
+    <row r="66" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A66" s="11" t="s">
         <v>99</v>
       </c>
@@ -3247,11 +3238,11 @@
       <c r="D66" s="11" t="s">
         <v>114</v>
       </c>
-      <c r="E66" s="17"/>
-      <c r="F66" s="17"/>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A67" s="16" t="s">
+      <c r="E66" s="16"/>
+      <c r="F66" s="16"/>
+    </row>
+    <row r="67" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A67" s="15" t="s">
         <v>102</v>
       </c>
       <c r="B67" s="11" t="s">
@@ -3263,56 +3254,56 @@
       <c r="D67" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="E67" s="17"/>
-      <c r="F67" s="17"/>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A68" s="16" t="s">
+      <c r="E67" s="16"/>
+      <c r="F67" s="16"/>
+    </row>
+    <row r="68" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A68" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="B68" s="16">
-        <v>0</v>
-      </c>
-      <c r="C68" s="16" t="s">
+      <c r="B68" s="15">
+        <v>0</v>
+      </c>
+      <c r="C68" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="D68" s="16" t="s">
+      <c r="D68" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="E68" s="17"/>
-      <c r="F68" s="17"/>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A69" s="16" t="s">
+      <c r="E68" s="16"/>
+      <c r="F68" s="16"/>
+    </row>
+    <row r="69" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A69" s="15" t="s">
         <v>102</v>
       </c>
       <c r="B69">
         <v>0</v>
       </c>
-      <c r="C69" s="16" t="s">
+      <c r="C69" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="D69" s="16" t="s">
+      <c r="D69" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="E69" s="17"/>
-      <c r="F69" s="17"/>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="E70" s="17"/>
-      <c r="F70" s="17"/>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="E71" s="17"/>
-      <c r="F71" s="17"/>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A72" s="17"/>
-      <c r="B72" s="17"/>
-      <c r="C72" s="17"/>
-      <c r="D72" s="17"/>
-      <c r="E72" s="17"/>
-      <c r="F72" s="17"/>
+      <c r="E69" s="16"/>
+      <c r="F69" s="16"/>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E70" s="16"/>
+      <c r="F70" s="16"/>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E71" s="16"/>
+      <c r="F71" s="16"/>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A72" s="16"/>
+      <c r="B72" s="16"/>
+      <c r="C72" s="16"/>
+      <c r="D72" s="16"/>
+      <c r="E72" s="16"/>
+      <c r="F72" s="16"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3323,9 +3314,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -3333,7 +3324,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -3341,7 +3332,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -3349,7 +3340,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -3365,13 +3356,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:B10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="37.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="37.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -3379,75 +3370,75 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="B2" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B2" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B3" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="B4" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B4" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B5" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="B6" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B6" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="B7" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B7" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="B8" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B8" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="B9" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B9" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="B10" s="15">
+      <c r="B10" s="14">
         <v>1</v>
       </c>
     </row>
@@ -3459,12 +3450,12 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>18</v>
       </c>
@@ -3472,27 +3463,27 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="B2" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B2" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="B3" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B3" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="B4" s="15">
+      <c r="B4" s="14">
         <v>1</v>
       </c>
     </row>

</xml_diff>